<commit_message>
Design site category A reference buildings
</commit_message>
<xml_diff>
--- a/casestudy_structures/casestudy__S_alpha_values_for_design.xlsx
+++ b/casestudy_structures/casestudy__S_alpha_values_for_design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hsuhhde-my.sharepoint.com/personal/clemettn_hsu_hamburg/Documents/01_arbeit/14_PhD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\clemettn\Documents\phd\casestudy_structures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{3EF92303-2A83-43A9-820D-7790CA7EBF03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4418256-F92F-43EE-B450-50F8BBE30067}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAB7950-B6B7-4DCC-A610-053E93FC09CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="0" windowWidth="14790" windowHeight="11370" xr2:uid="{DC730AE3-3318-4566-B7B3-9327F9026A54}"/>
+    <workbookView xWindow="30825" yWindow="810" windowWidth="21600" windowHeight="11295" xr2:uid="{DC730AE3-3318-4566-B7B3-9327F9026A54}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,28 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="16">
   <si>
     <t>[g]</t>
   </si>
   <si>
     <t>[m/s²]</t>
-  </si>
-  <si>
-    <r>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="subscript"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-      </rPr>
-      <t>α,c</t>
-    </r>
   </si>
   <si>
     <r>
@@ -159,6 +143,41 @@
       </rPr>
       <t xml:space="preserve"> &gt;</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>α,A</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="subscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>α,C</t>
+    </r>
+  </si>
+  <si>
+    <t>&lt;-- Soil Class A</t>
   </si>
 </sst>
 </file>
@@ -589,288 +608,485 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C936370-7B7D-47D6-AC6A-0502C8F0FCEA}">
-  <dimension ref="C2:K18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="C2:K33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="3:11" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="C2" t="s">
+    <row r="2" spans="3:11" ht="18" x14ac:dyDescent="0.35">
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
         <v>3</v>
-      </c>
-      <c r="D2" s="3">
-        <v>1.456</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="3" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C3" t="s">
-        <v>4</v>
       </c>
       <c r="D3" s="3">
         <v>9.81</v>
       </c>
       <c r="E3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="3:11" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
       <c r="D4" s="3"/>
       <c r="I4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J4">
         <v>1.3</v>
       </c>
       <c r="K4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="3:11" s="5" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="C5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="9"/>
-      <c r="F5" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="G5" s="9"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="3:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="I5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J5">
         <v>3.25</v>
       </c>
       <c r="K5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C6" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
       <c r="I6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J6">
         <v>6.5</v>
       </c>
       <c r="K6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" ht="18" x14ac:dyDescent="0.35">
+      <c r="C9" s="9" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C7" s="3">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6">
-        <f>C7/$D$3</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="7">
-        <f>D7*$D$2</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="4">
-        <f t="shared" ref="G7:G16" si="0">F7*9.81</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C8" s="3">
+      <c r="D9" s="9"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="9"/>
+      <c r="H9" t="s">
+        <v>2</v>
+      </c>
+      <c r="I9" s="3">
+        <v>1.456</v>
+      </c>
+      <c r="J9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="6">
-        <f t="shared" ref="D8:D16" si="1">C8/$D$3</f>
+      <c r="D10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="6">
+        <f>C11/$D$3</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="7">
+        <f>D11*$I$9</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <f>F11*$D$3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C12" s="3">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6">
+        <f t="shared" ref="D12:D20" si="0">C12/$D$3</f>
         <v>0.1019367991845056</v>
       </c>
-      <c r="F8" s="7">
-        <f t="shared" ref="F8:F16" si="2">D8*$D$2</f>
+      <c r="F12" s="7">
+        <f>D12*$I$9</f>
         <v>0.14841997961264014</v>
       </c>
-      <c r="G8" s="4">
-        <f>F8*9.81</f>
+      <c r="G12" s="4">
+        <f t="shared" ref="G12:G20" si="1">F12*$D$3</f>
         <v>1.456</v>
       </c>
     </row>
-    <row r="9" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C9" s="3">
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C13" s="3">
         <v>2</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D13" s="6">
+        <f t="shared" si="0"/>
+        <v>0.2038735983690112</v>
+      </c>
+      <c r="F13" s="7">
+        <f>D13*$I$9</f>
+        <v>0.29683995922528028</v>
+      </c>
+      <c r="G13" s="4">
         <f t="shared" si="1"/>
+        <v>2.9119999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C14" s="3">
+        <v>3</v>
+      </c>
+      <c r="D14" s="6">
+        <f t="shared" si="0"/>
+        <v>0.3058103975535168</v>
+      </c>
+      <c r="F14" s="7">
+        <f>D14*$I$9</f>
+        <v>0.44525993883792042</v>
+      </c>
+      <c r="G14" s="4">
+        <f t="shared" si="1"/>
+        <v>4.3679999999999994</v>
+      </c>
+    </row>
+    <row r="15" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C15" s="3">
+        <v>4</v>
+      </c>
+      <c r="D15" s="6">
+        <f t="shared" si="0"/>
+        <v>0.4077471967380224</v>
+      </c>
+      <c r="F15" s="7">
+        <f>D15*$I$9</f>
+        <v>0.59367991845056056</v>
+      </c>
+      <c r="G15" s="4">
+        <f t="shared" si="1"/>
+        <v>5.8239999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C16" s="3">
+        <v>5</v>
+      </c>
+      <c r="D16" s="6">
+        <f t="shared" si="0"/>
+        <v>0.509683995922528</v>
+      </c>
+      <c r="F16" s="7">
+        <f>D16*$I$9</f>
+        <v>0.74209989806320076</v>
+      </c>
+      <c r="G16" s="4">
+        <f t="shared" si="1"/>
+        <v>7.28</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C17" s="3">
+        <v>6</v>
+      </c>
+      <c r="D17" s="6">
+        <f t="shared" si="0"/>
+        <v>0.6116207951070336</v>
+      </c>
+      <c r="F17" s="7">
+        <f>D17*$I$9</f>
+        <v>0.89051987767584084</v>
+      </c>
+      <c r="G17" s="4">
+        <f t="shared" si="1"/>
+        <v>8.7359999999999989</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C18" s="3">
+        <v>7</v>
+      </c>
+      <c r="D18" s="6">
+        <f t="shared" si="0"/>
+        <v>0.7135575942915392</v>
+      </c>
+      <c r="F18" s="7">
+        <f>D18*$I$9</f>
+        <v>1.0389398572884812</v>
+      </c>
+      <c r="G18" s="4">
+        <f t="shared" si="1"/>
+        <v>10.192</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C19" s="3">
+        <v>10</v>
+      </c>
+      <c r="D19" s="6">
+        <f t="shared" si="0"/>
+        <v>1.019367991845056</v>
+      </c>
+      <c r="F19" s="7">
+        <f>D19*$I$9</f>
+        <v>1.4841997961264015</v>
+      </c>
+      <c r="G19" s="4">
+        <f t="shared" si="1"/>
+        <v>14.56</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C20" s="3">
+        <v>12</v>
+      </c>
+      <c r="D20" s="6">
+        <f t="shared" si="0"/>
+        <v>1.2232415902140672</v>
+      </c>
+      <c r="F20" s="7">
+        <f>D20*$I$9</f>
+        <v>1.7810397553516817</v>
+      </c>
+      <c r="G20" s="4">
+        <f t="shared" si="1"/>
+        <v>17.471999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="3:11" ht="18" x14ac:dyDescent="0.35">
+      <c r="C22" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="F22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="9"/>
+      <c r="H22" t="s">
+        <v>2</v>
+      </c>
+      <c r="I22" s="6">
+        <v>1</v>
+      </c>
+      <c r="J22" t="s">
+        <v>15</v>
+      </c>
+      <c r="K22" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="3">
+        <v>0</v>
+      </c>
+      <c r="D24" s="6">
+        <f>C24/$D$3</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="7">
+        <f>D11*$I$22</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <f>F24*$D$3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="3">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0.13</v>
+      </c>
+      <c r="F25" s="7">
+        <f>D12*$I$22</f>
+        <v>0.1019367991845056</v>
+      </c>
+      <c r="G25" s="4">
+        <f t="shared" ref="G25:G33" si="2">F25*$D$3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C26" s="3">
+        <v>2</v>
+      </c>
+      <c r="D26" s="6">
+        <f t="shared" ref="D25:D33" si="3">C26/$D$3</f>
         <v>0.2038735983690112</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F26" s="7">
+        <f>D13*$I$22</f>
+        <v>0.2038735983690112</v>
+      </c>
+      <c r="G26" s="4">
         <f t="shared" si="2"/>
-        <v>0.29683995922528028</v>
-      </c>
-      <c r="G9" s="4">
-        <f t="shared" si="0"/>
-        <v>2.9119999999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C10" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C27" s="3">
         <v>3</v>
       </c>
-      <c r="D10" s="6">
-        <f t="shared" si="1"/>
+      <c r="D27" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="F27" s="7">
+        <f>D14*$I$22</f>
         <v>0.3058103975535168</v>
       </c>
-      <c r="F10" s="7">
+      <c r="G27" s="4">
         <f t="shared" si="2"/>
-        <v>0.44525993883792042</v>
-      </c>
-      <c r="G10" s="4">
-        <f t="shared" si="0"/>
-        <v>4.3679999999999994</v>
-      </c>
-    </row>
-    <row r="11" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C11" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C28" s="3">
         <v>4</v>
       </c>
-      <c r="D11" s="6">
-        <f t="shared" si="1"/>
+      <c r="D28" s="6">
+        <v>0.4</v>
+      </c>
+      <c r="F28" s="7">
+        <f>D15*$I$22</f>
         <v>0.4077471967380224</v>
       </c>
-      <c r="F11" s="7">
+      <c r="G28" s="4">
         <f t="shared" si="2"/>
-        <v>0.59367991845056056</v>
-      </c>
-      <c r="G11" s="4">
-        <f>F11*9.81</f>
-        <v>5.8239999999999998</v>
-      </c>
-    </row>
-    <row r="12" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C12" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C29" s="3">
         <v>5</v>
       </c>
-      <c r="D12" s="6">
-        <f t="shared" si="1"/>
+      <c r="D29" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="F29" s="7">
+        <f>D16*$I$22</f>
         <v>0.509683995922528</v>
       </c>
-      <c r="F12" s="7">
+      <c r="G29" s="4">
         <f t="shared" si="2"/>
-        <v>0.74209989806320076</v>
-      </c>
-      <c r="G12" s="4">
-        <f t="shared" si="0"/>
-        <v>7.28</v>
-      </c>
-    </row>
-    <row r="13" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C13" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C30" s="3">
         <v>6</v>
       </c>
-      <c r="D13" s="6">
-        <f t="shared" si="1"/>
+      <c r="D30" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="F30" s="7">
+        <f>D17*$I$22</f>
         <v>0.6116207951070336</v>
       </c>
-      <c r="F13" s="7">
-        <f>D13*$D$2</f>
-        <v>0.89051987767584084</v>
-      </c>
-      <c r="G13" s="4">
-        <f t="shared" si="0"/>
-        <v>8.7359999999999989</v>
-      </c>
-    </row>
-    <row r="14" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C14" s="3">
+      <c r="G30" s="4">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C31" s="3">
         <v>7</v>
       </c>
-      <c r="D14" s="6">
-        <f t="shared" si="1"/>
+      <c r="D31" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="F31" s="7">
+        <f>D18*$I$22</f>
         <v>0.7135575942915392</v>
       </c>
-      <c r="F14" s="7">
+      <c r="G31" s="4">
         <f t="shared" si="2"/>
-        <v>1.0389398572884812</v>
-      </c>
-      <c r="G14" s="4">
-        <f t="shared" si="0"/>
-        <v>10.192</v>
-      </c>
-    </row>
-    <row r="15" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C15" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C32" s="3">
         <v>10</v>
       </c>
-      <c r="D15" s="6">
-        <f t="shared" si="1"/>
+      <c r="D32" s="6">
+        <v>1</v>
+      </c>
+      <c r="F32" s="7">
+        <f>D19*$I$22</f>
         <v>1.019367991845056</v>
       </c>
-      <c r="F15" s="7">
+      <c r="G32" s="4">
         <f t="shared" si="2"/>
-        <v>1.4841997961264015</v>
-      </c>
-      <c r="G15" s="4">
-        <f t="shared" si="0"/>
-        <v>14.56</v>
-      </c>
-    </row>
-    <row r="16" spans="3:11" x14ac:dyDescent="0.35">
-      <c r="C16" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C33" s="3">
         <v>12</v>
       </c>
-      <c r="D16" s="6">
-        <f t="shared" si="1"/>
+      <c r="D33" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="F33" s="7">
+        <f>D20*$I$22</f>
         <v>1.2232415902140672</v>
       </c>
-      <c r="F16" s="7">
+      <c r="G33" s="4">
         <f t="shared" si="2"/>
-        <v>1.7810397553516817</v>
-      </c>
-      <c r="G16" s="4">
-        <f t="shared" si="0"/>
-        <v>17.471999999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.35">
-      <c r="C17" s="3"/>
-      <c r="D17" s="6"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.35">
-      <c r="C18" s="3"/>
-      <c r="D18" s="6"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="4"/>
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="C5:D5"/>
+  <mergeCells count="4">
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="C22:D22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>